<commit_message>
fix tasks 1-4: correct split pricing, add task1+task2 notebooks, fix task4 cost calc
</commit_message>
<xml_diff>
--- a/assignment_01.xlsx
+++ b/assignment_01.xlsx
@@ -547,7 +547,7 @@
         <v>97</v>
       </c>
       <c r="J2" t="n">
-        <v>6.400000000000001e-05</v>
+        <v>1.542e-05</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         <v>101</v>
       </c>
       <c r="J3" t="n">
-        <v>6.48e-05</v>
+        <v>1.578e-05</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         <v>98</v>
       </c>
       <c r="J4" t="n">
-        <v>6.36e-05</v>
+        <v>1.542e-05</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         <v>97</v>
       </c>
       <c r="J5" t="n">
-        <v>6.340000000000001e-05</v>
+        <v>1.533e-05</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         <v>117</v>
       </c>
       <c r="J6" t="n">
-        <v>6.52e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         <v>117</v>
       </c>
       <c r="J7" t="n">
-        <v>6.52e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         <v>111</v>
       </c>
       <c r="J8" t="n">
-        <v>6.8e-05</v>
+        <v>1.686e-05</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v>114</v>
       </c>
       <c r="J9" t="n">
-        <v>6.740000000000001e-05</v>
+        <v>1.695e-05</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         <v>97</v>
       </c>
       <c r="J10" t="n">
-        <v>6.180000000000001e-05</v>
+        <v>1.509e-05</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>109</v>
       </c>
       <c r="J11" t="n">
-        <v>6.600000000000001e-05</v>
+        <v>1.644e-05</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
         <v>124</v>
       </c>
       <c r="J12" t="n">
-        <v>6.720000000000001e-05</v>
+        <v>1.752e-05</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1449,7 +1449,7 @@
         <v>114</v>
       </c>
       <c r="J13" t="n">
-        <v>6.660000000000001e-05</v>
+        <v>1.683e-05</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1531,7 +1531,7 @@
         <v>116</v>
       </c>
       <c r="J14" t="n">
-        <v>6.780000000000001e-05</v>
+        <v>1.713e-05</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         <v>80</v>
       </c>
       <c r="J15" t="n">
-        <v>5.84e-05</v>
+        <v>1.356e-05</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1695,7 +1695,7 @@
         <v>109</v>
       </c>
       <c r="J16" t="n">
-        <v>6.400000000000001e-05</v>
+        <v>1.614e-05</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         <v>117</v>
       </c>
       <c r="J17" t="n">
-        <v>6.8e-05</v>
+        <v>1.722e-05</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
         <v>124</v>
       </c>
       <c r="J18" t="n">
-        <v>7.04e-05</v>
+        <v>1.8e-05</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1941,7 +1941,7 @@
         <v>95</v>
       </c>
       <c r="J19" t="n">
-        <v>6.180000000000001e-05</v>
+        <v>1.497e-05</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
         <v>107</v>
       </c>
       <c r="J20" t="n">
-        <v>6.440000000000001e-05</v>
+        <v>1.608e-05</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2105,7 +2105,7 @@
         <v>99</v>
       </c>
       <c r="J21" t="n">
-        <v>6.26e-05</v>
+        <v>1.533e-05</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         <v>114</v>
       </c>
       <c r="J22" t="n">
-        <v>6.52e-05</v>
+        <v>1.662e-05</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -2269,7 +2269,7 @@
         <v>103</v>
       </c>
       <c r="J23" t="n">
-        <v>6.32e-05</v>
+        <v>1.566e-05</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         <v>103</v>
       </c>
       <c r="J24" t="n">
-        <v>6.380000000000001e-05</v>
+        <v>1.575e-05</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         <v>91</v>
       </c>
       <c r="J25" t="n">
-        <v>5.98e-05</v>
+        <v>1.443e-05</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         <v>105</v>
       </c>
       <c r="J26" t="n">
-        <v>6.3e-05</v>
+        <v>1.575e-05</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         <v>110</v>
       </c>
       <c r="J27" t="n">
-        <v>6.380000000000001e-05</v>
+        <v>1.617e-05</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         <v>113</v>
       </c>
       <c r="J28" t="n">
-        <v>6.560000000000001e-05</v>
+        <v>1.662e-05</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -2761,7 +2761,7 @@
         <v>107</v>
       </c>
       <c r="J29" t="n">
-        <v>6.3e-05</v>
+        <v>1.587e-05</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -2843,7 +2843,7 @@
         <v>106</v>
       </c>
       <c r="J30" t="n">
-        <v>6.380000000000001e-05</v>
+        <v>1.593e-05</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
         <v>111</v>
       </c>
       <c r="J31" t="n">
-        <v>6.42e-05</v>
+        <v>1.629e-05</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -3007,7 +3007,7 @@
         <v>117</v>
       </c>
       <c r="J32" t="n">
-        <v>6.720000000000001e-05</v>
+        <v>1.71e-05</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -3089,7 +3089,7 @@
         <v>112</v>
       </c>
       <c r="J33" t="n">
-        <v>6.52e-05</v>
+        <v>1.65e-05</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -3171,7 +3171,7 @@
         <v>108</v>
       </c>
       <c r="J34" t="n">
-        <v>6.560000000000001e-05</v>
+        <v>1.632e-05</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -3253,7 +3253,7 @@
         <v>109</v>
       </c>
       <c r="J35" t="n">
-        <v>6.400000000000001e-05</v>
+        <v>1.614e-05</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
         <v>105</v>
       </c>
       <c r="J36" t="n">
-        <v>6.32e-05</v>
+        <v>1.578e-05</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -3417,7 +3417,7 @@
         <v>101</v>
       </c>
       <c r="J37" t="n">
-        <v>6.36e-05</v>
+        <v>1.56e-05</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -3499,7 +3499,7 @@
         <v>110</v>
       </c>
       <c r="J38" t="n">
-        <v>6.48e-05</v>
+        <v>1.632e-05</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -3581,7 +3581,7 @@
         <v>130</v>
       </c>
       <c r="J39" t="n">
-        <v>7.2e-05</v>
+        <v>1.86e-05</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -3663,7 +3663,7 @@
         <v>96</v>
       </c>
       <c r="J40" t="n">
-        <v>6.14e-05</v>
+        <v>1.497e-05</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -3745,7 +3745,7 @@
         <v>117</v>
       </c>
       <c r="J41" t="n">
-        <v>6.560000000000001e-05</v>
+        <v>1.686e-05</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -3827,7 +3827,7 @@
         <v>107</v>
       </c>
       <c r="J42" t="n">
-        <v>6.400000000000001e-05</v>
+        <v>1.602e-05</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
         <v>84</v>
       </c>
       <c r="J43" t="n">
-        <v>5.9e-05</v>
+        <v>1.389e-05</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -3991,7 +3991,7 @@
         <v>101</v>
       </c>
       <c r="J44" t="n">
-        <v>6.3e-05</v>
+        <v>1.551e-05</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
         <v>113</v>
       </c>
       <c r="J45" t="n">
-        <v>6.86e-05</v>
+        <v>1.707e-05</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -4155,7 +4155,7 @@
         <v>105</v>
       </c>
       <c r="J46" t="n">
-        <v>6.58e-05</v>
+        <v>1.617e-05</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         <v>108</v>
       </c>
       <c r="J47" t="n">
-        <v>6.560000000000001e-05</v>
+        <v>1.632e-05</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         <v>104</v>
       </c>
       <c r="J48" t="n">
-        <v>6.52e-05</v>
+        <v>1.602e-05</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -4401,7 +4401,7 @@
         <v>130</v>
       </c>
       <c r="J49" t="n">
-        <v>7.240000000000001e-05</v>
+        <v>1.866e-05</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
         <v>103</v>
       </c>
       <c r="J50" t="n">
-        <v>6.48e-05</v>
+        <v>1.59e-05</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -4565,7 +4565,7 @@
         <v>106</v>
       </c>
       <c r="J51" t="n">
-        <v>6.660000000000001e-05</v>
+        <v>1.635e-05</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>

</xml_diff>